<commit_message>
Finished adding 2014 cotton data
</commit_message>
<xml_diff>
--- a/Data/2015_F013B4_CO_ISOS/2015_F013B4_CO_ISOS_CropCanopy.xlsx
+++ b/Data/2015_F013B4_CO_ISOS/2015_F013B4_CO_ISOS_CropCanopy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mnt\Data1\USDA-ALARC\GIS\PDI project\cottondata\Data\2015_F013B4_CO_ISOS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACC1DA50-DABE-4138-9D16-4716D7A1AD24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EF24D96-9DA7-4CDD-81FA-11FBD1F7647E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-1665" yWindow="-28410" windowWidth="18105" windowHeight="16065" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16200" yWindow="-28725" windowWidth="18105" windowHeight="14355" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Height" sheetId="11" r:id="rId1"/>
@@ -2242,18 +2242,6 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="10" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2263,7 +2251,16 @@
     <xf numFmtId="15" fontId="18" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="10" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2276,10 +2273,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="16" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="16" fontId="16" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2288,8 +2285,11 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="16" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2299,6 +2299,22 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="46" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="15" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2312,22 +2328,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="46" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -11036,6 +11036,10 @@
         <f>AVERAGE(F8:H11)/1.5</f>
         <v>11.222222222222221</v>
       </c>
+      <c r="L8" s="81">
+        <f>AVERAGE(F8:H11)/(1.5*1.016)</f>
+        <v>11.045494313210847</v>
+      </c>
       <c r="N8" s="114" t="s">
         <v>153</v>
       </c>
@@ -11062,6 +11066,7 @@
       <c r="H9" s="95">
         <v>18</v>
       </c>
+      <c r="L9" s="81"/>
       <c r="N9" s="114" t="s">
         <v>152</v>
       </c>
@@ -11082,6 +11087,7 @@
       <c r="H10" s="95">
         <v>17</v>
       </c>
+      <c r="L10" s="81"/>
     </row>
     <row r="11" spans="1:15" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="94"/>
@@ -11099,6 +11105,7 @@
       <c r="H11" s="92">
         <v>18</v>
       </c>
+      <c r="L11" s="81"/>
     </row>
     <row r="12" spans="1:15" ht="33" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B12" s="105" t="s">
@@ -11129,6 +11136,10 @@
       <c r="K12" s="101">
         <f>AVERAGE(F12:H15)/1.5</f>
         <v>10.944444444444445</v>
+      </c>
+      <c r="L12" s="81">
+        <f>AVERAGE(F12:H15)/(1.5*1.016)</f>
+        <v>10.772090988626422</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="33" customHeight="1" x14ac:dyDescent="0.25">
@@ -11149,6 +11160,7 @@
       <c r="H13" s="95">
         <v>16</v>
       </c>
+      <c r="L13" s="81"/>
     </row>
     <row r="14" spans="1:15" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="99"/>
@@ -11166,6 +11178,7 @@
       <c r="H14" s="95">
         <v>17</v>
       </c>
+      <c r="L14" s="81"/>
     </row>
     <row r="15" spans="1:15" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="94"/>
@@ -11183,6 +11196,7 @@
       <c r="H15" s="92">
         <v>15</v>
       </c>
+      <c r="L15" s="81"/>
     </row>
     <row r="16" spans="1:15" ht="33" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B16" s="109" t="s">
@@ -11214,8 +11228,12 @@
         <f>AVERAGE(F16:H19)/1.5</f>
         <v>10.111111111111111</v>
       </c>
-    </row>
-    <row r="17" spans="2:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L16" s="81">
+        <f>AVERAGE(F16:H19)/(1.5*1.016)</f>
+        <v>9.9518810148731411</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="112">
         <v>42151</v>
       </c>
@@ -11233,8 +11251,9 @@
       <c r="H17" s="95">
         <v>16</v>
       </c>
-    </row>
-    <row r="18" spans="2:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L17" s="81"/>
+    </row>
+    <row r="18" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="106"/>
       <c r="C18" s="106"/>
       <c r="D18" s="106"/>
@@ -11250,8 +11269,9 @@
       <c r="H18" s="95">
         <v>10</v>
       </c>
-    </row>
-    <row r="19" spans="2:11" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L18" s="81"/>
+    </row>
+    <row r="19" spans="2:12" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="106"/>
       <c r="C19" s="106"/>
       <c r="D19" s="106"/>
@@ -11267,8 +11287,9 @@
       <c r="H19" s="92">
         <v>16</v>
       </c>
-    </row>
-    <row r="20" spans="2:11" ht="33" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="L19" s="81"/>
+    </row>
+    <row r="20" spans="2:12" ht="33" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B20" s="109" t="s">
         <v>2</v>
       </c>
@@ -11298,8 +11319,12 @@
         <f>AVERAGE(F20:H23)/1.5</f>
         <v>10.222222222222223</v>
       </c>
-    </row>
-    <row r="21" spans="2:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L20" s="81">
+        <f>AVERAGE(F20:H23)/(1.5*1.016)</f>
+        <v>10.061242344706912</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="112">
         <v>42151</v>
       </c>
@@ -11317,8 +11342,9 @@
       <c r="H21" s="95">
         <v>16</v>
       </c>
-    </row>
-    <row r="22" spans="2:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L21" s="81"/>
+    </row>
+    <row r="22" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="106"/>
       <c r="C22" s="106"/>
       <c r="D22" s="106"/>
@@ -11334,8 +11360,9 @@
       <c r="H22" s="95">
         <v>18</v>
       </c>
-    </row>
-    <row r="23" spans="2:11" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L22" s="81"/>
+    </row>
+    <row r="23" spans="2:12" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="106"/>
       <c r="C23" s="106"/>
       <c r="D23" s="106"/>
@@ -11351,8 +11378,9 @@
       <c r="H23" s="92">
         <v>16</v>
       </c>
-    </row>
-    <row r="24" spans="2:11" ht="33" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="L23" s="81"/>
+    </row>
+    <row r="24" spans="2:12" ht="33" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B24" s="105" t="s">
         <v>2</v>
       </c>
@@ -11382,8 +11410,12 @@
         <f>AVERAGE(F24:H27)/1.5</f>
         <v>9.9444444444444446</v>
       </c>
-    </row>
-    <row r="25" spans="2:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L24" s="81">
+        <f>AVERAGE(F24:H27)/(1.5*1.016)</f>
+        <v>9.787839020122485</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="112">
         <v>42151</v>
       </c>
@@ -11401,8 +11433,9 @@
       <c r="H25" s="95">
         <v>17</v>
       </c>
-    </row>
-    <row r="26" spans="2:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L25" s="81"/>
+    </row>
+    <row r="26" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="99"/>
       <c r="C26" s="99"/>
       <c r="D26" s="94"/>
@@ -11418,8 +11451,9 @@
       <c r="H26" s="95">
         <v>14</v>
       </c>
-    </row>
-    <row r="27" spans="2:11" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L26" s="81"/>
+    </row>
+    <row r="27" spans="2:12" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="94"/>
       <c r="C27" s="94"/>
       <c r="D27" s="94"/>
@@ -11435,8 +11469,9 @@
       <c r="H27" s="92">
         <v>13</v>
       </c>
-    </row>
-    <row r="28" spans="2:11" ht="33" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="L27" s="81"/>
+    </row>
+    <row r="28" spans="2:12" ht="33" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B28" s="105" t="s">
         <v>3</v>
       </c>
@@ -11466,8 +11501,12 @@
         <f>AVERAGE(F28:H31)/1.5</f>
         <v>10.277777777777777</v>
       </c>
-    </row>
-    <row r="29" spans="2:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L28" s="81">
+        <f>AVERAGE(F28:H31)/(1.5*1.016)</f>
+        <v>10.115923009623797</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="100">
         <v>42150</v>
       </c>
@@ -11485,8 +11524,9 @@
       <c r="H29" s="95">
         <v>19</v>
       </c>
-    </row>
-    <row r="30" spans="2:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L29" s="81"/>
+    </row>
+    <row r="30" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="94"/>
       <c r="C30" s="94"/>
       <c r="D30" s="94"/>
@@ -11502,8 +11542,9 @@
       <c r="H30" s="111">
         <v>16</v>
       </c>
-    </row>
-    <row r="31" spans="2:11" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L30" s="81"/>
+    </row>
+    <row r="31" spans="2:12" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="94"/>
       <c r="C31" s="94"/>
       <c r="D31" s="94"/>
@@ -11519,8 +11560,9 @@
       <c r="H31" s="92">
         <v>17</v>
       </c>
-    </row>
-    <row r="32" spans="2:11" ht="33" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="L31" s="81"/>
+    </row>
+    <row r="32" spans="2:12" ht="33" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B32" s="109" t="s">
         <v>3</v>
       </c>
@@ -11549,6 +11591,10 @@
       <c r="K32" s="101">
         <f>AVERAGE(F32:H35)/1.5</f>
         <v>10.777777777777779</v>
+      </c>
+      <c r="L32" s="81">
+        <f>AVERAGE(F32:H35)/(1.5*1.016)</f>
+        <v>10.608048993875766</v>
       </c>
     </row>
     <row r="33" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
@@ -11569,6 +11615,7 @@
       <c r="H33" s="95">
         <v>17</v>
       </c>
+      <c r="L33" s="81"/>
     </row>
     <row r="34" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="106"/>
@@ -11586,6 +11633,7 @@
       <c r="H34" s="95">
         <v>16</v>
       </c>
+      <c r="L34" s="81"/>
     </row>
     <row r="35" spans="2:12" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B35" s="106"/>
@@ -11603,6 +11651,7 @@
       <c r="H35" s="92">
         <v>17</v>
       </c>
+      <c r="L35" s="81"/>
     </row>
     <row r="36" spans="2:12" ht="33" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B36" s="109" t="s">
@@ -11633,6 +11682,10 @@
       <c r="K36" s="101">
         <f>AVERAGE(F36:H39)/1.5</f>
         <v>9.6111111111111107</v>
+      </c>
+      <c r="L36" s="81">
+        <f>AVERAGE(F36:H39)/(1.5*1.016)</f>
+        <v>9.4597550306211726</v>
       </c>
     </row>
     <row r="37" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
@@ -11654,6 +11707,7 @@
         <v>14</v>
       </c>
       <c r="J37" s="107"/>
+      <c r="L37" s="81"/>
     </row>
     <row r="38" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="106"/>
@@ -11671,6 +11725,7 @@
       <c r="H38" s="95">
         <v>15</v>
       </c>
+      <c r="L38" s="81"/>
     </row>
     <row r="39" spans="2:12" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B39" s="106"/>
@@ -11688,6 +11743,7 @@
       <c r="H39" s="92">
         <v>15</v>
       </c>
+      <c r="L39" s="81"/>
     </row>
     <row r="40" spans="2:12" ht="33" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B40" s="105" t="s">
@@ -11718,6 +11774,10 @@
       <c r="K40" s="101">
         <f>AVERAGE(F40:H43)/1.5</f>
         <v>9.7777777777777768</v>
+      </c>
+      <c r="L40" s="81">
+        <f>AVERAGE(F40:H43)/(1.5*1.016)</f>
+        <v>9.6237970253718288</v>
       </c>
     </row>
     <row r="41" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
@@ -11738,6 +11798,7 @@
       <c r="H41" s="95">
         <v>16</v>
       </c>
+      <c r="L41" s="81"/>
     </row>
     <row r="42" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="94"/>
@@ -11755,6 +11816,7 @@
       <c r="H42" s="95">
         <v>15</v>
       </c>
+      <c r="L42" s="81"/>
     </row>
     <row r="43" spans="2:12" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B43" s="94"/>
@@ -11772,6 +11834,7 @@
       <c r="H43" s="92">
         <v>18</v>
       </c>
+      <c r="L43" s="81"/>
     </row>
     <row r="44" spans="2:12" ht="33" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B44" s="105" t="s">
@@ -11802,6 +11865,10 @@
       <c r="K44" s="101">
         <f>AVERAGE(F44:H47)/1.5</f>
         <v>8.7777777777777768</v>
+      </c>
+      <c r="L44" s="81">
+        <f>AVERAGE(F44:H47)/(1.5*1.016)</f>
+        <v>8.6395450568678918</v>
       </c>
     </row>
     <row r="45" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
@@ -11822,6 +11889,7 @@
       <c r="H45" s="97">
         <v>13</v>
       </c>
+      <c r="L45" s="81"/>
     </row>
     <row r="46" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="94"/>
@@ -11839,6 +11907,7 @@
       <c r="H46" s="95">
         <v>14</v>
       </c>
+      <c r="L46" s="81"/>
     </row>
     <row r="47" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="94"/>
@@ -11856,6 +11925,7 @@
       <c r="H47" s="92">
         <v>7</v>
       </c>
+      <c r="L47" s="81"/>
     </row>
     <row r="48" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="91"/>
@@ -11869,7 +11939,7 @@
         <f>AVERAGE(K44,K40,K36,K32,K28,K24,K20,K16,K12,K8)</f>
         <v>10.166666666666666</v>
       </c>
-      <c r="L48">
+      <c r="L48" s="81">
         <f>K48/1.02</f>
         <v>9.9673202614379086</v>
       </c>
@@ -15073,75 +15143,75 @@
       <c r="D6" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="182">
+      <c r="E6" s="180">
         <v>42192</v>
       </c>
-      <c r="F6" s="183"/>
-      <c r="G6" s="177">
+      <c r="F6" s="181"/>
+      <c r="G6" s="183">
         <v>42198</v>
       </c>
-      <c r="H6" s="178"/>
-      <c r="I6" s="182">
+      <c r="H6" s="184"/>
+      <c r="I6" s="180">
         <v>42207</v>
       </c>
-      <c r="J6" s="183"/>
-      <c r="K6" s="177">
+      <c r="J6" s="181"/>
+      <c r="K6" s="183">
         <v>42212</v>
       </c>
-      <c r="L6" s="178"/>
-      <c r="M6" s="177">
+      <c r="L6" s="184"/>
+      <c r="M6" s="183">
         <v>42219</v>
       </c>
-      <c r="N6" s="178"/>
-      <c r="O6" s="177">
+      <c r="N6" s="184"/>
+      <c r="O6" s="183">
         <v>42227</v>
       </c>
-      <c r="P6" s="178"/>
-      <c r="Q6" s="177">
+      <c r="P6" s="184"/>
+      <c r="Q6" s="183">
         <v>42240</v>
       </c>
-      <c r="R6" s="178"/>
-      <c r="S6" s="177">
+      <c r="R6" s="184"/>
+      <c r="S6" s="183">
         <v>42255</v>
       </c>
-      <c r="T6" s="178"/>
+      <c r="T6" s="184"/>
     </row>
     <row r="7" spans="1:29" ht="15" x14ac:dyDescent="0.25">
       <c r="D7" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="184">
+      <c r="E7" s="182">
         <v>188</v>
       </c>
-      <c r="F7" s="183"/>
-      <c r="G7" s="179">
+      <c r="F7" s="181"/>
+      <c r="G7" s="185">
         <v>194</v>
       </c>
-      <c r="H7" s="178"/>
-      <c r="I7" s="184">
+      <c r="H7" s="184"/>
+      <c r="I7" s="182">
         <v>203</v>
       </c>
-      <c r="J7" s="183"/>
-      <c r="K7" s="179">
+      <c r="J7" s="181"/>
+      <c r="K7" s="185">
         <v>208</v>
       </c>
-      <c r="L7" s="178"/>
-      <c r="M7" s="179">
+      <c r="L7" s="184"/>
+      <c r="M7" s="185">
         <v>215</v>
       </c>
-      <c r="N7" s="178"/>
-      <c r="O7" s="179">
+      <c r="N7" s="184"/>
+      <c r="O7" s="185">
         <v>223</v>
       </c>
-      <c r="P7" s="178"/>
-      <c r="Q7" s="179">
+      <c r="P7" s="184"/>
+      <c r="Q7" s="185">
         <v>236</v>
       </c>
-      <c r="R7" s="178"/>
-      <c r="S7" s="179">
+      <c r="R7" s="184"/>
+      <c r="S7" s="185">
         <v>251</v>
       </c>
-      <c r="T7" s="178"/>
+      <c r="T7" s="184"/>
     </row>
     <row r="8" spans="1:29" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D8" s="10"/>
@@ -15169,14 +15239,14 @@
         <v>221</v>
       </c>
       <c r="P8" s="153"/>
-      <c r="Q8" s="180" t="s">
+      <c r="Q8" s="186" t="s">
         <v>221</v>
       </c>
-      <c r="R8" s="181"/>
-      <c r="S8" s="180" t="s">
+      <c r="R8" s="187"/>
+      <c r="S8" s="186" t="s">
         <v>221</v>
       </c>
-      <c r="T8" s="181"/>
+      <c r="T8" s="187"/>
       <c r="V8" s="82" t="s">
         <v>220</v>
       </c>
@@ -19177,89 +19247,95 @@
       </c>
     </row>
     <row r="59" spans="2:29" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E59" s="185" t="s">
+      <c r="E59" s="177" t="s">
         <v>212</v>
       </c>
-      <c r="F59" s="186"/>
+      <c r="F59" s="178"/>
       <c r="G59" s="138"/>
-      <c r="I59" s="185" t="s">
+      <c r="I59" s="177" t="s">
         <v>212</v>
       </c>
-      <c r="J59" s="186"/>
-      <c r="O59" s="185" t="s">
+      <c r="J59" s="178"/>
+      <c r="O59" s="177" t="s">
         <v>211</v>
       </c>
-      <c r="P59" s="186"/>
-      <c r="Q59" s="185"/>
-      <c r="R59" s="186"/>
+      <c r="P59" s="178"/>
+      <c r="Q59" s="177"/>
+      <c r="R59" s="178"/>
     </row>
     <row r="60" spans="2:29" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E60" s="187"/>
-      <c r="F60" s="187"/>
+      <c r="E60" s="179"/>
+      <c r="F60" s="179"/>
       <c r="G60" s="138"/>
-      <c r="I60" s="187"/>
-      <c r="J60" s="187"/>
-      <c r="O60" s="187"/>
-      <c r="P60" s="187"/>
-      <c r="Q60" s="187"/>
-      <c r="R60" s="187"/>
+      <c r="I60" s="179"/>
+      <c r="J60" s="179"/>
+      <c r="O60" s="179"/>
+      <c r="P60" s="179"/>
+      <c r="Q60" s="179"/>
+      <c r="R60" s="179"/>
     </row>
     <row r="61" spans="2:29" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E61" s="187"/>
-      <c r="F61" s="187"/>
+      <c r="E61" s="179"/>
+      <c r="F61" s="179"/>
       <c r="G61" s="138"/>
-      <c r="I61" s="187"/>
-      <c r="J61" s="187"/>
-      <c r="O61" s="187"/>
-      <c r="P61" s="187"/>
-      <c r="Q61" s="187"/>
-      <c r="R61" s="187"/>
+      <c r="I61" s="179"/>
+      <c r="J61" s="179"/>
+      <c r="O61" s="179"/>
+      <c r="P61" s="179"/>
+      <c r="Q61" s="179"/>
+      <c r="R61" s="179"/>
     </row>
     <row r="62" spans="2:29" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E62" s="187"/>
-      <c r="F62" s="187"/>
+      <c r="E62" s="179"/>
+      <c r="F62" s="179"/>
       <c r="G62" s="138"/>
-      <c r="I62" s="187"/>
-      <c r="J62" s="187"/>
-      <c r="O62" s="187"/>
-      <c r="P62" s="187"/>
-      <c r="Q62" s="187"/>
-      <c r="R62" s="187"/>
+      <c r="I62" s="179"/>
+      <c r="J62" s="179"/>
+      <c r="O62" s="179"/>
+      <c r="P62" s="179"/>
+      <c r="Q62" s="179"/>
+      <c r="R62" s="179"/>
     </row>
     <row r="63" spans="2:29" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E63" s="166"/>
-      <c r="F63" s="166"/>
-      <c r="I63" s="166"/>
-      <c r="J63" s="166"/>
-      <c r="O63" s="166"/>
-      <c r="P63" s="166"/>
-      <c r="Q63" s="166"/>
-      <c r="R63" s="166"/>
+      <c r="E63" s="165"/>
+      <c r="F63" s="165"/>
+      <c r="I63" s="165"/>
+      <c r="J63" s="165"/>
+      <c r="O63" s="165"/>
+      <c r="P63" s="165"/>
+      <c r="Q63" s="165"/>
+      <c r="R63" s="165"/>
     </row>
     <row r="64" spans="2:29" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E64" s="166"/>
-      <c r="F64" s="166"/>
-      <c r="I64" s="166"/>
-      <c r="J64" s="166"/>
-      <c r="O64" s="166"/>
-      <c r="P64" s="166"/>
-      <c r="Q64" s="166"/>
-      <c r="R64" s="166"/>
+      <c r="E64" s="165"/>
+      <c r="F64" s="165"/>
+      <c r="I64" s="165"/>
+      <c r="J64" s="165"/>
+      <c r="O64" s="165"/>
+      <c r="P64" s="165"/>
+      <c r="Q64" s="165"/>
+      <c r="R64" s="165"/>
     </row>
     <row r="65" spans="15:18" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="O65" s="166"/>
-      <c r="P65" s="166"/>
-      <c r="Q65" s="166"/>
-      <c r="R65" s="166"/>
+      <c r="O65" s="165"/>
+      <c r="P65" s="165"/>
+      <c r="Q65" s="165"/>
+      <c r="R65" s="165"/>
     </row>
     <row r="66" spans="15:18" x14ac:dyDescent="0.2">
-      <c r="O66" s="166"/>
-      <c r="P66" s="166"/>
-      <c r="Q66" s="166"/>
-      <c r="R66" s="166"/>
+      <c r="O66" s="165"/>
+      <c r="P66" s="165"/>
+      <c r="Q66" s="165"/>
+      <c r="R66" s="165"/>
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="Q8:R8"/>
+    <mergeCell ref="S8:T8"/>
+    <mergeCell ref="Q6:R6"/>
+    <mergeCell ref="Q7:R7"/>
     <mergeCell ref="Q59:R66"/>
     <mergeCell ref="O59:P66"/>
     <mergeCell ref="E6:F6"/>
@@ -19276,12 +19352,6 @@
     <mergeCell ref="M7:N7"/>
     <mergeCell ref="I6:J6"/>
     <mergeCell ref="I7:J7"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="Q8:R8"/>
-    <mergeCell ref="S8:T8"/>
-    <mergeCell ref="Q6:R6"/>
-    <mergeCell ref="Q7:R7"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0" footer="0.3"/>
   <pageSetup scale="69" fitToHeight="2" orientation="portrait" r:id="rId1"/>
@@ -25732,59 +25802,59 @@
       <c r="C5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O5" s="161"/>
-      <c r="P5" s="162"/>
+      <c r="O5" s="157"/>
+      <c r="P5" s="158"/>
     </row>
     <row r="6" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E6" s="165" t="s">
+      <c r="E6" s="164" t="s">
         <v>58</v>
       </c>
-      <c r="F6" s="166"/>
-      <c r="O6" s="162"/>
-      <c r="P6" s="162"/>
+      <c r="F6" s="165"/>
+      <c r="O6" s="158"/>
+      <c r="P6" s="158"/>
     </row>
     <row r="7" spans="1:28" ht="15" x14ac:dyDescent="0.25">
       <c r="D7" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="163">
+      <c r="E7" s="159">
         <v>42157</v>
       </c>
-      <c r="F7" s="158"/>
-      <c r="G7" s="167">
+      <c r="F7" s="160"/>
+      <c r="G7" s="166">
         <v>42170</v>
       </c>
-      <c r="H7" s="168"/>
-      <c r="I7" s="159">
+      <c r="H7" s="167"/>
+      <c r="I7" s="162">
         <v>42184</v>
       </c>
-      <c r="J7" s="158"/>
-      <c r="K7" s="159">
+      <c r="J7" s="160"/>
+      <c r="K7" s="162">
         <v>42198</v>
       </c>
-      <c r="L7" s="158"/>
-      <c r="M7" s="159">
+      <c r="L7" s="160"/>
+      <c r="M7" s="162">
         <v>42212</v>
       </c>
-      <c r="N7" s="158"/>
-      <c r="O7" s="159">
+      <c r="N7" s="160"/>
+      <c r="O7" s="162">
         <v>42227</v>
       </c>
-      <c r="P7" s="158"/>
-      <c r="Q7" s="159">
+      <c r="P7" s="160"/>
+      <c r="Q7" s="162">
         <v>42243</v>
       </c>
-      <c r="R7" s="158"/>
-      <c r="S7" s="159">
+      <c r="R7" s="160"/>
+      <c r="S7" s="162">
         <v>42255</v>
       </c>
-      <c r="T7" s="158"/>
-      <c r="U7" s="157"/>
-      <c r="V7" s="158"/>
-      <c r="W7" s="157"/>
-      <c r="X7" s="158"/>
-      <c r="Y7" s="157"/>
-      <c r="Z7" s="158"/>
+      <c r="T7" s="160"/>
+      <c r="U7" s="168"/>
+      <c r="V7" s="160"/>
+      <c r="W7" s="168"/>
+      <c r="X7" s="160"/>
+      <c r="Y7" s="168"/>
+      <c r="Z7" s="160"/>
       <c r="AA7" s="29"/>
       <c r="AB7" s="29"/>
     </row>
@@ -25792,44 +25862,44 @@
       <c r="D8" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="E8" s="164">
+      <c r="E8" s="161">
         <v>153</v>
       </c>
-      <c r="F8" s="158"/>
+      <c r="F8" s="160"/>
       <c r="G8" s="64">
         <v>166</v>
       </c>
       <c r="H8" s="64"/>
-      <c r="I8" s="157">
+      <c r="I8" s="168">
         <v>180</v>
       </c>
-      <c r="J8" s="158"/>
-      <c r="K8" s="160">
+      <c r="J8" s="160"/>
+      <c r="K8" s="163">
         <v>194</v>
       </c>
-      <c r="L8" s="158"/>
-      <c r="M8" s="160">
+      <c r="L8" s="160"/>
+      <c r="M8" s="163">
         <v>208</v>
       </c>
-      <c r="N8" s="158"/>
-      <c r="O8" s="160">
+      <c r="N8" s="160"/>
+      <c r="O8" s="163">
         <v>223</v>
       </c>
-      <c r="P8" s="158"/>
-      <c r="Q8" s="160">
+      <c r="P8" s="160"/>
+      <c r="Q8" s="163">
         <v>236</v>
       </c>
-      <c r="R8" s="158"/>
-      <c r="S8" s="160">
+      <c r="R8" s="160"/>
+      <c r="S8" s="163">
         <v>251</v>
       </c>
-      <c r="T8" s="158"/>
-      <c r="U8" s="157"/>
-      <c r="V8" s="158"/>
-      <c r="W8" s="157"/>
-      <c r="X8" s="158"/>
-      <c r="Y8" s="157"/>
-      <c r="Z8" s="158"/>
+      <c r="T8" s="160"/>
+      <c r="U8" s="168"/>
+      <c r="V8" s="160"/>
+      <c r="W8" s="168"/>
+      <c r="X8" s="160"/>
+      <c r="Y8" s="168"/>
+      <c r="Z8" s="160"/>
       <c r="AA8" s="29"/>
       <c r="AB8" s="29"/>
     </row>
@@ -29316,6 +29386,16 @@
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="W7:X7"/>
+    <mergeCell ref="W8:X8"/>
+    <mergeCell ref="Y7:Z7"/>
+    <mergeCell ref="Y8:Z8"/>
+    <mergeCell ref="Q7:R7"/>
+    <mergeCell ref="Q8:R8"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="S8:T8"/>
+    <mergeCell ref="U7:V7"/>
+    <mergeCell ref="U8:V8"/>
     <mergeCell ref="O5:P6"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="E8:F8"/>
@@ -29329,16 +29409,6 @@
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="I7:J7"/>
     <mergeCell ref="I8:J8"/>
-    <mergeCell ref="W7:X7"/>
-    <mergeCell ref="W8:X8"/>
-    <mergeCell ref="Y7:Z7"/>
-    <mergeCell ref="Y8:Z8"/>
-    <mergeCell ref="Q7:R7"/>
-    <mergeCell ref="Q8:R8"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="S8:T8"/>
-    <mergeCell ref="U7:V7"/>
-    <mergeCell ref="U8:V8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -29381,7 +29451,7 @@
       <c r="O3" s="155" t="s">
         <v>62</v>
       </c>
-      <c r="P3" s="169"/>
+      <c r="P3" s="173"/>
     </row>
     <row r="4" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
@@ -29389,7 +29459,7 @@
       </c>
       <c r="C4" s="4"/>
       <c r="O4" s="156"/>
-      <c r="P4" s="169"/>
+      <c r="P4" s="173"/>
     </row>
     <row r="5" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="4"/>
@@ -29397,7 +29467,7 @@
         <v>44</v>
       </c>
       <c r="O5" s="156"/>
-      <c r="P5" s="169"/>
+      <c r="P5" s="173"/>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.2">
       <c r="C6" s="65"/>
@@ -29405,7 +29475,7 @@
         <v>45</v>
       </c>
       <c r="O6" s="156"/>
-      <c r="P6" s="169"/>
+      <c r="P6" s="173"/>
     </row>
     <row r="7" spans="1:28" ht="15" x14ac:dyDescent="0.25">
       <c r="D7" s="10" t="s">
@@ -29414,43 +29484,43 @@
       <c r="E7" s="69">
         <v>42157</v>
       </c>
-      <c r="F7" s="171" t="s">
+      <c r="F7" s="170" t="s">
         <v>59</v>
       </c>
-      <c r="G7" s="159">
+      <c r="G7" s="162">
         <v>42170</v>
       </c>
-      <c r="H7" s="158"/>
-      <c r="I7" s="159">
+      <c r="H7" s="160"/>
+      <c r="I7" s="162">
         <v>42184</v>
       </c>
-      <c r="J7" s="170"/>
-      <c r="K7" s="159">
+      <c r="J7" s="172"/>
+      <c r="K7" s="162">
         <v>42198</v>
       </c>
-      <c r="L7" s="170"/>
-      <c r="M7" s="159">
+      <c r="L7" s="172"/>
+      <c r="M7" s="162">
         <v>42212</v>
       </c>
-      <c r="N7" s="158"/>
-      <c r="O7" s="159">
+      <c r="N7" s="160"/>
+      <c r="O7" s="162">
         <v>42227</v>
       </c>
-      <c r="P7" s="158"/>
-      <c r="Q7" s="159">
+      <c r="P7" s="160"/>
+      <c r="Q7" s="162">
         <v>42243</v>
       </c>
-      <c r="R7" s="158"/>
-      <c r="S7" s="159">
+      <c r="R7" s="160"/>
+      <c r="S7" s="162">
         <v>42255</v>
       </c>
-      <c r="T7" s="158"/>
-      <c r="U7" s="157"/>
-      <c r="V7" s="158"/>
-      <c r="W7" s="157"/>
-      <c r="X7" s="158"/>
-      <c r="Y7" s="157"/>
-      <c r="Z7" s="158"/>
+      <c r="T7" s="160"/>
+      <c r="U7" s="168"/>
+      <c r="V7" s="160"/>
+      <c r="W7" s="168"/>
+      <c r="X7" s="160"/>
+      <c r="Y7" s="168"/>
+      <c r="Z7" s="160"/>
       <c r="AA7" s="29"/>
       <c r="AB7" s="29"/>
     </row>
@@ -29461,41 +29531,41 @@
       <c r="E8" s="33">
         <v>153</v>
       </c>
-      <c r="F8" s="172"/>
-      <c r="G8" s="157">
+      <c r="F8" s="171"/>
+      <c r="G8" s="168">
         <v>166</v>
       </c>
-      <c r="H8" s="158"/>
-      <c r="I8" s="157">
+      <c r="H8" s="160"/>
+      <c r="I8" s="168">
         <v>180</v>
       </c>
-      <c r="J8" s="173"/>
-      <c r="K8" s="157">
+      <c r="J8" s="169"/>
+      <c r="K8" s="168">
         <v>194</v>
       </c>
-      <c r="L8" s="173"/>
-      <c r="M8" s="160">
+      <c r="L8" s="169"/>
+      <c r="M8" s="163">
         <v>208</v>
       </c>
-      <c r="N8" s="158"/>
-      <c r="O8" s="160">
+      <c r="N8" s="160"/>
+      <c r="O8" s="163">
         <v>223</v>
       </c>
-      <c r="P8" s="158"/>
-      <c r="Q8" s="160">
+      <c r="P8" s="160"/>
+      <c r="Q8" s="163">
         <v>236</v>
       </c>
-      <c r="R8" s="158"/>
-      <c r="S8" s="160">
+      <c r="R8" s="160"/>
+      <c r="S8" s="163">
         <v>251</v>
       </c>
-      <c r="T8" s="158"/>
-      <c r="U8" s="157"/>
-      <c r="V8" s="158"/>
-      <c r="W8" s="157"/>
-      <c r="X8" s="158"/>
-      <c r="Y8" s="157"/>
-      <c r="Z8" s="158"/>
+      <c r="T8" s="160"/>
+      <c r="U8" s="168"/>
+      <c r="V8" s="160"/>
+      <c r="W8" s="168"/>
+      <c r="X8" s="160"/>
+      <c r="Y8" s="168"/>
+      <c r="Z8" s="160"/>
       <c r="AA8" s="29"/>
       <c r="AB8" s="29"/>
     </row>
@@ -32559,37 +32629,37 @@
       <c r="E65" s="69">
         <v>42157</v>
       </c>
-      <c r="F65" s="171" t="s">
+      <c r="F65" s="170" t="s">
         <v>59</v>
       </c>
-      <c r="G65" s="159">
+      <c r="G65" s="162">
         <v>42170</v>
       </c>
-      <c r="H65" s="158"/>
-      <c r="I65" s="159">
+      <c r="H65" s="160"/>
+      <c r="I65" s="162">
         <v>42184</v>
       </c>
-      <c r="J65" s="170"/>
-      <c r="K65" s="159">
+      <c r="J65" s="172"/>
+      <c r="K65" s="162">
         <v>42198</v>
       </c>
-      <c r="L65" s="170"/>
-      <c r="M65" s="159">
+      <c r="L65" s="172"/>
+      <c r="M65" s="162">
         <v>42212</v>
       </c>
-      <c r="N65" s="158"/>
-      <c r="O65" s="159">
+      <c r="N65" s="160"/>
+      <c r="O65" s="162">
         <v>42227</v>
       </c>
-      <c r="P65" s="158"/>
-      <c r="Q65" s="159">
+      <c r="P65" s="160"/>
+      <c r="Q65" s="162">
         <v>42243</v>
       </c>
-      <c r="R65" s="158"/>
-      <c r="S65" s="159">
+      <c r="R65" s="160"/>
+      <c r="S65" s="162">
         <v>42255</v>
       </c>
-      <c r="T65" s="158"/>
+      <c r="T65" s="160"/>
     </row>
     <row r="66" spans="4:20" ht="15" x14ac:dyDescent="0.25">
       <c r="D66" s="10" t="s">
@@ -32598,53 +32668,44 @@
       <c r="E66" s="33">
         <v>153</v>
       </c>
-      <c r="F66" s="172"/>
-      <c r="G66" s="157">
+      <c r="F66" s="171"/>
+      <c r="G66" s="168">
         <v>166</v>
       </c>
-      <c r="H66" s="158"/>
-      <c r="I66" s="157">
+      <c r="H66" s="160"/>
+      <c r="I66" s="168">
         <v>180</v>
       </c>
-      <c r="J66" s="173"/>
-      <c r="K66" s="157">
+      <c r="J66" s="169"/>
+      <c r="K66" s="168">
         <v>194</v>
       </c>
-      <c r="L66" s="173"/>
-      <c r="M66" s="160">
+      <c r="L66" s="169"/>
+      <c r="M66" s="163">
         <v>208</v>
       </c>
-      <c r="N66" s="158"/>
-      <c r="O66" s="160">
+      <c r="N66" s="160"/>
+      <c r="O66" s="163">
         <v>223</v>
       </c>
-      <c r="P66" s="158"/>
-      <c r="Q66" s="160">
+      <c r="P66" s="160"/>
+      <c r="Q66" s="163">
         <v>236</v>
       </c>
-      <c r="R66" s="158"/>
-      <c r="S66" s="160">
+      <c r="R66" s="160"/>
+      <c r="S66" s="163">
         <v>251</v>
       </c>
-      <c r="T66" s="158"/>
+      <c r="T66" s="160"/>
     </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="O65:P65"/>
-    <mergeCell ref="Q65:R65"/>
-    <mergeCell ref="S65:T65"/>
-    <mergeCell ref="G66:H66"/>
-    <mergeCell ref="I66:J66"/>
-    <mergeCell ref="K66:L66"/>
-    <mergeCell ref="M66:N66"/>
-    <mergeCell ref="O66:P66"/>
-    <mergeCell ref="Q66:R66"/>
-    <mergeCell ref="S66:T66"/>
-    <mergeCell ref="F65:F66"/>
-    <mergeCell ref="G65:H65"/>
-    <mergeCell ref="I65:J65"/>
-    <mergeCell ref="K65:L65"/>
-    <mergeCell ref="M65:N65"/>
+    <mergeCell ref="O8:P8"/>
+    <mergeCell ref="O3:P6"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="M7:N7"/>
     <mergeCell ref="F7:F8"/>
     <mergeCell ref="Y8:Z8"/>
     <mergeCell ref="Q7:R7"/>
@@ -32661,12 +32722,21 @@
     <mergeCell ref="I8:J8"/>
     <mergeCell ref="K8:L8"/>
     <mergeCell ref="M8:N8"/>
-    <mergeCell ref="O8:P8"/>
-    <mergeCell ref="O3:P6"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="F65:F66"/>
+    <mergeCell ref="G65:H65"/>
+    <mergeCell ref="I65:J65"/>
+    <mergeCell ref="K65:L65"/>
+    <mergeCell ref="M65:N65"/>
+    <mergeCell ref="O65:P65"/>
+    <mergeCell ref="Q65:R65"/>
+    <mergeCell ref="S65:T65"/>
+    <mergeCell ref="G66:H66"/>
+    <mergeCell ref="I66:J66"/>
+    <mergeCell ref="K66:L66"/>
+    <mergeCell ref="M66:N66"/>
+    <mergeCell ref="O66:P66"/>
+    <mergeCell ref="Q66:R66"/>
+    <mergeCell ref="S66:T66"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>